<commit_message>
Nivel 0: compensaciones internas + control de matches (cada match = 0)
</commit_message>
<xml_diff>
--- a/data/raw/banco_beta_202603.xlsx
+++ b/data/raw/banco_beta_202603.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="238">
   <si>
     <t>Fecha</t>
   </si>
@@ -97,13 +97,13 @@
     <t>DEBITO TRANSFERENCIA A ENVASES DEL PLATA SRL</t>
   </si>
   <si>
-    <t>ACREDITACION COMERCIO FISERV QR LOTE 3229</t>
-  </si>
-  <si>
     <t>ACREDITACION COMERCIO FISERV QR LOTE</t>
   </si>
   <si>
-    <t>1906</t>
+    <t>3229</t>
+  </si>
+  <si>
+    <t>ACREDITACION COMERCIO FISERV QR LOTE 1906</t>
   </si>
   <si>
     <t>4673</t>
@@ -124,13 +124,13 @@
     <t>ACREDITACION COMERCIO FISERV QR LOTE 9937</t>
   </si>
   <si>
-    <t>2894</t>
+    <t>ACREDITACION COMERCIO FISERV QR LOTE 2894</t>
   </si>
   <si>
     <t>DEBITO TRANSFERENCIA A ENERGIA URBANA SA</t>
   </si>
   <si>
-    <t>6262</t>
+    <t>ACREDITACION COMERCIO FISERV QR LOTE 6262</t>
   </si>
   <si>
     <t>ACREDITACION COMERCIO FISERV QR LOTE 9749</t>
@@ -154,13 +154,31 @@
     <t>ACREDITACION COMERCIO FISERV QR LOTE 9773</t>
   </si>
   <si>
-    <t>ACREDITACION COMERCIO FISERV QR LOTE 8864</t>
-  </si>
-  <si>
-    <t>ACREDITACION COMERCIO FISERV QR LOTE 5060</t>
-  </si>
-  <si>
-    <t>DEBITO TRANSFERENCIA A LIMPIEZA TOTAL SA</t>
+    <t>8864</t>
+  </si>
+  <si>
+    <t>5060</t>
+  </si>
+  <si>
+    <t>DEBITO TRANSFERENCIA A LIMPIEZA TOTAL</t>
+  </si>
+  <si>
+    <t>SA</t>
+  </si>
+  <si>
+    <t>DEBITO TRANSFERENCIA A PAPELERA CENTRAL SRL</t>
+  </si>
+  <si>
+    <t>8094</t>
+  </si>
+  <si>
+    <t>DEBITO TRANSFERENCIA A SEGUROS</t>
+  </si>
+  <si>
+    <t>PROTECCION SA</t>
+  </si>
+  <si>
+    <t>1203</t>
   </si>
   <si>
     <t>DEBITO TRANSFERENCIA A PAPELERA</t>
@@ -169,31 +187,16 @@
     <t>CENTRAL SRL</t>
   </si>
   <si>
-    <t>ACREDITACION COMERCIO FISERV QR LOTE 8094</t>
-  </si>
-  <si>
-    <t>DEBITO TRANSFERENCIA A SEGUROS</t>
-  </si>
-  <si>
-    <t>PROTECCION SA</t>
-  </si>
-  <si>
-    <t>1203</t>
-  </si>
-  <si>
-    <t>DEBITO TRANSFERENCIA A PAPELERA CENTRAL SRL</t>
-  </si>
-  <si>
     <t>3338</t>
   </si>
   <si>
-    <t>1561</t>
-  </si>
-  <si>
-    <t>3523</t>
-  </si>
-  <si>
-    <t>8900</t>
+    <t>ACREDITACION COMERCIO FISERV QR LOTE 1561</t>
+  </si>
+  <si>
+    <t>ACREDITACION COMERCIO FISERV QR LOTE 3523</t>
+  </si>
+  <si>
+    <t>ACREDITACION COMERCIO FISERV QR LOTE 8900</t>
   </si>
   <si>
     <t>Nro Operación</t>
@@ -1067,13 +1070,13 @@
         <v>23</v>
       </c>
       <c r="C1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1084,13 +1087,13 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1101,13 +1104,13 @@
         <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1118,13 +1121,13 @@
         <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1135,38 +1138,26 @@
         <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
       <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" t="s">
-        <v>65</v>
-      </c>
-      <c r="D6" t="s">
-        <v>124</v>
-      </c>
-      <c r="E6" t="s">
-        <v>183</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
         <v>66</v>
@@ -1179,8 +1170,20 @@
       </c>
     </row>
     <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
       <c r="B8" t="s">
         <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E8" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1191,13 +1194,13 @@
         <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1205,16 +1208,16 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1230,13 +1233,13 @@
         <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E12" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1247,13 +1250,13 @@
         <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D13" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E13" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1264,13 +1267,13 @@
         <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D14" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E14" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1281,13 +1284,13 @@
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D15" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E15" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1298,13 +1301,13 @@
         <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E16" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1320,13 +1323,13 @@
         <v>35</v>
       </c>
       <c r="C18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E18" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1337,13 +1340,13 @@
         <v>25</v>
       </c>
       <c r="C19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D19" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E19" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1351,21 +1354,33 @@
         <v>7</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D20" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E20" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>7</v>
+      </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>25</v>
+      </c>
+      <c r="C21" t="s">
+        <v>78</v>
+      </c>
+      <c r="D21" t="s">
+        <v>137</v>
+      </c>
+      <c r="E21" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1373,16 +1388,16 @@
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="C22" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D22" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E22" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1390,33 +1405,33 @@
         <v>7</v>
       </c>
       <c r="B23" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E23" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B24" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="C24" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D24" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E24" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1424,72 +1439,84 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D25" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E25" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>9</v>
+      </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="C26" t="s">
+        <v>83</v>
+      </c>
+      <c r="D26" t="s">
+        <v>142</v>
+      </c>
+      <c r="E26" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B27" t="s">
         <v>25</v>
       </c>
       <c r="C27" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D27" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="E27" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C28" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D28" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="E28" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B29" t="s">
         <v>25</v>
       </c>
       <c r="C29" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D29" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E29" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -1497,84 +1524,84 @@
         <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C30" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D30" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E30" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B31" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="C31" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D31" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="E31" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B32" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="C32" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D32" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="E32" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C33" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D33" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E33" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B34" t="s">
         <v>25</v>
       </c>
       <c r="C34" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D34" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="E34" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -1582,50 +1609,50 @@
         <v>12</v>
       </c>
       <c r="B35" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C35" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D35" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E35" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B36" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="C36" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D36" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E36" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="C37" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D37" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E37" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -1633,50 +1660,38 @@
         <v>13</v>
       </c>
       <c r="B38" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C38" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D38" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E38" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" t="s">
-        <v>13</v>
-      </c>
       <c r="B39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C39" t="s">
-        <v>93</v>
-      </c>
-      <c r="D39" t="s">
-        <v>152</v>
-      </c>
-      <c r="E39" t="s">
-        <v>211</v>
+        <v>34</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B40" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C40" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D40" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E40" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -1684,50 +1699,38 @@
         <v>14</v>
       </c>
       <c r="B41" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C41" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D41" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E41" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C42" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D42" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E42" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" t="s">
-        <v>15</v>
-      </c>
       <c r="B43" t="s">
         <v>46</v>
-      </c>
-      <c r="C43" t="s">
-        <v>97</v>
-      </c>
-      <c r="D43" t="s">
-        <v>156</v>
-      </c>
-      <c r="E43" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -1738,13 +1741,13 @@
         <v>25</v>
       </c>
       <c r="C44" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D44" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E44" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -1752,33 +1755,21 @@
         <v>16</v>
       </c>
       <c r="B45" t="s">
+        <v>27</v>
+      </c>
+      <c r="C45" t="s">
+        <v>100</v>
+      </c>
+      <c r="D45" t="s">
+        <v>159</v>
+      </c>
+      <c r="E45" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="B46" t="s">
         <v>47</v>
-      </c>
-      <c r="C45" t="s">
-        <v>99</v>
-      </c>
-      <c r="D45" t="s">
-        <v>158</v>
-      </c>
-      <c r="E45" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5">
-      <c r="A46" t="s">
-        <v>16</v>
-      </c>
-      <c r="B46" t="s">
-        <v>25</v>
-      </c>
-      <c r="C46" t="s">
-        <v>100</v>
-      </c>
-      <c r="D46" t="s">
-        <v>159</v>
-      </c>
-      <c r="E46" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -1786,7 +1777,7 @@
         <v>16</v>
       </c>
       <c r="B47" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="C47" t="s">
         <v>101</v>
@@ -1803,7 +1794,7 @@
         <v>16</v>
       </c>
       <c r="B48" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C48" t="s">
         <v>102</v>
@@ -1817,15 +1808,15 @@
     </row>
     <row r="49" spans="1:5">
       <c r="B49" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B50" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C50" t="s">
         <v>103</v>
@@ -1842,7 +1833,7 @@
         <v>17</v>
       </c>
       <c r="B51" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C51" t="s">
         <v>104</v>
@@ -1855,33 +1846,33 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" t="s">
+      <c r="B52" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53" t="s">
         <v>17</v>
       </c>
-      <c r="B52" t="s">
-        <v>52</v>
-      </c>
-      <c r="C52" t="s">
+      <c r="B53" t="s">
+        <v>25</v>
+      </c>
+      <c r="C53" t="s">
         <v>105</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D53" t="s">
         <v>164</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E53" t="s">
         <v>223</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5">
-      <c r="B53" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B54" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="C54" t="s">
         <v>106</v>
@@ -1895,7 +1886,7 @@
     </row>
     <row r="55" spans="1:5">
       <c r="B55" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -1903,7 +1894,7 @@
         <v>18</v>
       </c>
       <c r="B56" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C56" t="s">
         <v>107</v>
@@ -1916,25 +1907,25 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" t="s">
+      <c r="B57" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" t="s">
         <v>18</v>
       </c>
-      <c r="B57" t="s">
-        <v>33</v>
-      </c>
-      <c r="C57" t="s">
+      <c r="B58" t="s">
+        <v>25</v>
+      </c>
+      <c r="C58" t="s">
         <v>108</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D58" t="s">
         <v>167</v>
       </c>
-      <c r="E57" t="s">
+      <c r="E58" t="s">
         <v>226</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5">
-      <c r="B58" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -1942,7 +1933,7 @@
         <v>18</v>
       </c>
       <c r="B59" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="C59" t="s">
         <v>109</v>
@@ -1955,59 +1946,47 @@
       </c>
     </row>
     <row r="60" spans="1:5">
-      <c r="A60" t="s">
-        <v>19</v>
-      </c>
       <c r="B60" t="s">
-        <v>28</v>
-      </c>
-      <c r="C60" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" t="s">
+        <v>18</v>
+      </c>
+      <c r="B61" t="s">
+        <v>55</v>
+      </c>
+      <c r="C61" t="s">
         <v>110</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D61" t="s">
         <v>169</v>
       </c>
-      <c r="E60" t="s">
+      <c r="E61" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
-      <c r="B61" t="s">
+    <row r="62" spans="1:5">
+      <c r="B62" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5">
-      <c r="A62" t="s">
-        <v>19</v>
-      </c>
-      <c r="B62" t="s">
-        <v>25</v>
-      </c>
-      <c r="C62" t="s">
-        <v>111</v>
-      </c>
-      <c r="D62" t="s">
-        <v>170</v>
-      </c>
-      <c r="E62" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B63" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C63" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D63" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E63" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -2017,19 +1996,19 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B65" t="s">
         <v>25</v>
       </c>
       <c r="C65" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D65" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E65" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -2037,29 +2016,41 @@
         <v>20</v>
       </c>
       <c r="B66" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="C66" t="s">
+        <v>113</v>
+      </c>
+      <c r="D66" t="s">
+        <v>172</v>
+      </c>
+      <c r="E66" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" t="s">
+        <v>20</v>
+      </c>
+      <c r="B67" t="s">
+        <v>25</v>
+      </c>
+      <c r="C67" t="s">
         <v>114</v>
       </c>
-      <c r="D66" t="s">
+      <c r="D67" t="s">
         <v>173</v>
       </c>
-      <c r="E66" t="s">
+      <c r="E67" t="s">
         <v>232</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5">
-      <c r="B67" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B68" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C68" t="s">
         <v>115</v>
@@ -2073,7 +2064,7 @@
     </row>
     <row r="69" spans="1:5">
       <c r="B69" t="s">
-        <v>58</v>
+        <v>34</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -2081,7 +2072,7 @@
         <v>21</v>
       </c>
       <c r="B70" t="s">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="C70" t="s">
         <v>116</v>
@@ -2095,10 +2086,10 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B71" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C71" t="s">
         <v>117</v>
@@ -2111,8 +2102,20 @@
       </c>
     </row>
     <row r="72" spans="1:5">
+      <c r="A72" t="s">
+        <v>22</v>
+      </c>
       <c r="B72" t="s">
-        <v>59</v>
+        <v>60</v>
+      </c>
+      <c r="C72" t="s">
+        <v>118</v>
+      </c>
+      <c r="D72" t="s">
+        <v>177</v>
+      </c>
+      <c r="E72" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -2123,13 +2126,13 @@
         <v>25</v>
       </c>
       <c r="C73" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D73" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E73" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>

</xml_diff>